<commit_message>
Add new orders to 16MAR2026 sheet: 546659, 546660, 546661, 546871, 546202, 546746
</commit_message>
<xml_diff>
--- a/shared/documents/ACS_Order_MAR2026_CS---3474f087-3bc7-4a73-92d1-7d4857b78eb3.xlsx
+++ b/shared/documents/ACS_Order_MAR2026_CS---3474f087-3bc7-4a73-92d1-7d4857b78eb3.xlsx
@@ -14066,116 +14066,294 @@
       </c>
     </row>
     <row r="7" ht="18" customFormat="1" customHeight="1" s="112">
-      <c r="B7" s="46" t="n"/>
-      <c r="C7" s="39" t="n"/>
-      <c r="D7" s="514" t="n"/>
-      <c r="E7" s="103" t="n"/>
-      <c r="F7" s="40" t="n"/>
-      <c r="G7" s="40" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>546659</t>
+        </is>
+      </c>
+      <c r="B7" s="46" t="n">
+        <v>0.5972222222222222</v>
+      </c>
+      <c r="C7" s="39" t="inlineStr">
+        <is>
+          <t>TST&gt;AP</t>
+        </is>
+      </c>
+      <c r="D7" s="514" t="inlineStr">
+        <is>
+          <t>WH9918 So蘇 60139929</t>
+        </is>
+      </c>
+      <c r="E7" s="103" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>0.6006944444444444</v>
+      </c>
+      <c r="G7" s="40" t="n">
+        <v>0.6215277777777778</v>
+      </c>
       <c r="H7" s="39" t="n"/>
       <c r="I7" s="438" t="n"/>
       <c r="J7" s="441" t="n"/>
-      <c r="K7" s="437" t="n"/>
-      <c r="L7" s="436" t="n"/>
+      <c r="K7" s="437" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="436" t="n">
+        <v>400</v>
+      </c>
       <c r="M7" s="437">
         <f>SUM(K7:L7)</f>
         <v/>
       </c>
-      <c r="N7" s="437" t="n"/>
+      <c r="N7" s="437" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="8" ht="18" customFormat="1" customHeight="1" s="112">
-      <c r="A8" s="45" t="n"/>
-      <c r="B8" s="46" t="n"/>
-      <c r="C8" s="365" t="n"/>
-      <c r="D8" s="366" t="n"/>
-      <c r="E8" s="170" t="n"/>
-      <c r="F8" s="487" t="n"/>
-      <c r="G8" s="516" t="n"/>
+      <c r="A8" s="45" t="inlineStr">
+        <is>
+          <t>546660</t>
+        </is>
+      </c>
+      <c r="B8" s="46" t="n">
+        <v>0.6180555555555556</v>
+      </c>
+      <c r="C8" s="365" t="inlineStr">
+        <is>
+          <t>MB509&gt;TST</t>
+        </is>
+      </c>
+      <c r="D8" s="366" t="inlineStr">
+        <is>
+          <t>WH9918 So蘇 60139929 / RN377 Abble 梁 95514488</t>
+        </is>
+      </c>
+      <c r="E8" s="170" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F8" s="390" t="n">
+        <v>0.6388888888888888</v>
+      </c>
+      <c r="G8" s="172" t="n">
+        <v>0.6597222222222222</v>
+      </c>
       <c r="H8" s="172" t="n"/>
       <c r="I8" s="172" t="n"/>
-      <c r="J8" s="516" t="n"/>
-      <c r="K8" s="517" t="n"/>
-      <c r="L8" s="507" t="n"/>
-      <c r="M8" s="488" t="n"/>
-      <c r="N8" s="489" t="n"/>
+      <c r="J8" s="516" t="inlineStr">
+        <is>
+          <t>P5 x 2</t>
+        </is>
+      </c>
+      <c r="K8" s="517" t="n">
+        <v>70</v>
+      </c>
+      <c r="L8" s="507" t="n">
+        <v>870</v>
+      </c>
+      <c r="M8" s="488">
+        <f>SUM(K8:L8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="489" t="n">
+        <v>60</v>
+      </c>
       <c r="O8" s="448" t="n"/>
       <c r="P8" s="448" t="n"/>
     </row>
     <row r="9" ht="18" customFormat="1" customHeight="1" s="112">
-      <c r="A9" s="45" t="n"/>
-      <c r="B9" s="46" t="n"/>
-      <c r="C9" s="39" t="n"/>
-      <c r="D9" s="440" t="n"/>
-      <c r="E9" s="39" t="n"/>
+      <c r="A9" s="45" t="inlineStr">
+        <is>
+          <t>546661</t>
+        </is>
+      </c>
+      <c r="B9" s="46" t="n">
+        <v>0.6597222222222222</v>
+      </c>
+      <c r="C9" s="39" t="inlineStr">
+        <is>
+          <t>TST&gt;AP</t>
+        </is>
+      </c>
+      <c r="D9" s="440" t="inlineStr">
+        <is>
+          <t>CT8022 Wong Jacky 69986953</t>
+        </is>
+      </c>
+      <c r="E9" s="39" t="inlineStr">
+        <is>
+          <t>No show</t>
+        </is>
+      </c>
       <c r="F9" s="40" t="n"/>
       <c r="G9" s="40" t="n"/>
       <c r="H9" s="39" t="n"/>
       <c r="I9" s="438" t="n"/>
       <c r="J9" s="441" t="n"/>
-      <c r="K9" s="437" t="n"/>
-      <c r="L9" s="436" t="n"/>
+      <c r="K9" s="437" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="436" t="n">
+        <v>400</v>
+      </c>
       <c r="M9" s="437">
         <f>SUM(K9:L9)</f>
         <v/>
       </c>
-      <c r="N9" s="437" t="n"/>
+      <c r="N9" s="437" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="45" t="n"/>
-      <c r="B10" s="48" t="n"/>
-      <c r="C10" s="39" t="n"/>
-      <c r="D10" s="167" t="n"/>
-      <c r="E10" s="39" t="n"/>
-      <c r="F10" s="40" t="n"/>
-      <c r="G10" s="40" t="n"/>
+      <c r="A10" s="45" t="inlineStr">
+        <is>
+          <t>546871</t>
+        </is>
+      </c>
+      <c r="B10" s="48" t="n">
+        <v>0.7708333333333334</v>
+      </c>
+      <c r="C10" s="39" t="inlineStr">
+        <is>
+          <t>TST&gt;AP</t>
+        </is>
+      </c>
+      <c r="D10" s="167" t="inlineStr">
+        <is>
+          <t>WH9918 So蘇 60139929</t>
+        </is>
+      </c>
+      <c r="E10" s="39" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F10" s="40" t="n">
+        <v>0.7729166666666667</v>
+      </c>
+      <c r="G10" s="40" t="n">
+        <v>0.7958333333333333</v>
+      </c>
       <c r="H10" s="449" t="n"/>
       <c r="I10" s="438" t="n"/>
       <c r="J10" s="441" t="n"/>
-      <c r="K10" s="437" t="n"/>
-      <c r="L10" s="436" t="n"/>
+      <c r="K10" s="437" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="436" t="n">
+        <v>400</v>
+      </c>
       <c r="M10" s="437">
         <f>SUM(K10:L10)</f>
         <v/>
       </c>
-      <c r="N10" s="437" t="n"/>
+      <c r="N10" s="437" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="45" t="n"/>
-      <c r="B11" s="48" t="n"/>
-      <c r="C11" s="39" t="n"/>
-      <c r="D11" s="48" t="n"/>
-      <c r="E11" s="39" t="n"/>
-      <c r="F11" s="40" t="n"/>
-      <c r="G11" s="40" t="n"/>
+      <c r="A11" s="45" t="inlineStr">
+        <is>
+          <t>546202</t>
+        </is>
+      </c>
+      <c r="B11" s="48" t="inlineStr">
+        <is>
+          <t>即時</t>
+        </is>
+      </c>
+      <c r="C11" s="39" t="inlineStr">
+        <is>
+          <t>AP&gt;旺角帝京</t>
+        </is>
+      </c>
+      <c r="D11" s="48" t="inlineStr">
+        <is>
+          <t>YW8506 Kelvin 陳師傅 +85291939799</t>
+        </is>
+      </c>
+      <c r="E11" s="39" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F11" s="40" t="n">
+        <v>0.8090277777777778</v>
+      </c>
+      <c r="G11" s="40" t="n">
+        <v>0.8368055555555556</v>
+      </c>
       <c r="H11" s="39" t="n"/>
       <c r="I11" s="438" t="n"/>
       <c r="J11" s="441" t="n"/>
-      <c r="K11" s="437" t="n"/>
-      <c r="L11" s="436" t="n"/>
+      <c r="K11" s="437" t="n">
+        <v>35</v>
+      </c>
+      <c r="L11" s="436" t="n">
+        <v>435</v>
+      </c>
       <c r="M11" s="437">
         <f>SUM(K11:L11)</f>
         <v/>
       </c>
-      <c r="N11" s="437" t="n"/>
+      <c r="N11" s="437" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="45" t="n"/>
-      <c r="B12" s="48" t="n"/>
-      <c r="C12" s="39" t="n"/>
-      <c r="D12" s="440" t="n"/>
-      <c r="E12" s="39" t="n"/>
-      <c r="F12" s="40" t="n"/>
-      <c r="G12" s="40" t="n"/>
+      <c r="A12" s="45" t="inlineStr">
+        <is>
+          <t>546746</t>
+        </is>
+      </c>
+      <c r="B12" s="48" t="n">
+        <v>0.9236111111111112</v>
+      </c>
+      <c r="C12" s="39" t="inlineStr">
+        <is>
+          <t>3v401&gt;Cordis</t>
+        </is>
+      </c>
+      <c r="D12" s="440" t="inlineStr">
+        <is>
+          <t>LJ9800 Stanley 梁師傅 +85298286100 / WW8421 Patrick 9318 2082</t>
+        </is>
+      </c>
+      <c r="E12" s="39" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F12" s="40" t="n">
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="G12" s="40" t="n">
+        <v>0.9652777777777778</v>
+      </c>
       <c r="H12" s="39" t="n"/>
       <c r="I12" s="438" t="n"/>
-      <c r="J12" s="441" t="n"/>
-      <c r="K12" s="437" t="n"/>
-      <c r="L12" s="436" t="n"/>
+      <c r="J12" s="441" t="inlineStr">
+        <is>
+          <t>P5 x 2</t>
+        </is>
+      </c>
+      <c r="K12" s="437" t="n">
+        <v>70</v>
+      </c>
+      <c r="L12" s="436" t="n">
+        <v>870</v>
+      </c>
       <c r="M12" s="437">
         <f>SUM(K12:L12)</f>
         <v/>
       </c>
-      <c r="N12" s="437" t="n"/>
+      <c r="N12" s="437" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="45" t="n"/>
@@ -15045,7 +15223,6 @@
           <t>14:55:00</t>
         </is>
       </c>
-      <c r="J135" t="inlineStr"/>
       <c r="K135" t="n">
         <v>0</v>
       </c>
@@ -15187,7 +15364,6 @@
           <t>No show</t>
         </is>
       </c>
-      <c r="J138" t="inlineStr"/>
       <c r="K138" t="n">
         <v>0</v>
       </c>
@@ -15235,7 +15411,6 @@
           <t>19:06:00</t>
         </is>
       </c>
-      <c r="J139" t="inlineStr"/>
       <c r="K139" t="n">
         <v>0</v>
       </c>

</xml_diff>